<commit_message>
feat: sync otomatis rombel, program, dan relasi siswa
- deriveProgramFromKelas untuk deteksi program dari nama rombel
- Cascade update/delete rombel ke students.kelas & elearning_setups
- Auto-set program siswa saat create/update berdasarkan kelas
- Rombel filter & combobox dikelompokan per program
- Syncronize bersihin relasi siswa non-AKTIF & rombel kosong
- cleanup: autoComplete, placeholder, monitoring initialLevel
</commit_message>
<xml_diff>
--- a/public/templates/format-upload-alumni.xlsx
+++ b/public/templates/format-upload-alumni.xlsx
@@ -1,40 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\PLCS\1PAND\PKBM\E-learning\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366603C4-1286-40C3-AD78-51CDCE16709D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15930" xr2:uid="{AD3937EE-34AA-448B-9943-4E2FDE8671D0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15930"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>No</t>
   </si>
@@ -67,6 +51,9 @@
   </si>
   <si>
     <t>Kecamatan</t>
+  </si>
+  <si>
+    <t>Kabupaten/ Kota</t>
   </si>
   <si>
     <t>Provinsi</t>
@@ -96,8 +83,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,24 +93,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -135,19 +119,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
     <border>
       <left style="thin">
         <color indexed="64"/>
@@ -161,37 +139,28 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{EB3A5341-0C68-486D-BB40-7B4DD1232412}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -200,10 +169,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -372,6 +341,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -398,24 +368,25 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -476,45 +447,40 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E79DCB5-B161-4A20-B3E8-396135C1A0E4}">
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.570313" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.710938" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.425781" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.42578" customWidth="1"/>
     <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="3.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="3.425781" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.425781" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.570313" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.85547" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.71094" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.855469" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="3.710938" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.42578" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.57031" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.42578" customWidth="1"/>
+    <col min="19" max="19" width="12.71094" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -572,8 +538,11 @@
       <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -593,8 +562,8 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(import): support custom password column in excel templates and import handlers
</commit_message>
<xml_diff>
--- a/public/templates/format-upload-alumni.xlsx
+++ b/public/templates/format-upload-alumni.xlsx
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>E-Mail</t>
+  </si>
+  <si>
+    <t>Password</t>
   </si>
   <si>
     <t>PROGRAM YANG DIAMBIL</t>
@@ -475,9 +478,10 @@
     <col min="14" max="14" width="3.710938" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="17.42578" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.57031" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.42578" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.42578" customWidth="1"/>
-    <col min="19" max="19" width="12.71094" customWidth="1"/>
+    <col min="19" max="19" width="16.14063" customWidth="1"/>
+    <col min="20" max="20" width="13.28516" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.5">
@@ -540,6 +544,9 @@
       </c>
       <c r="T1" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="2">
@@ -563,6 +570,7 @@
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>